<commit_message>
Web a la 2.8.0: capturas nuevas, guía, demo con todos los módulos y pago de Contable
- Capturas 2.8.0 (demo y lotes inventados): ejecución, revisión del lote,
  laboratorio, informe, analítica, herramientas.
- Home: «La interfaz» con 6 bloques; sin «score de integridad» (el informe
  cuenta, no puntúa); herramientas 9 / 7 en CORE y Contable.
- Guía a 2.8: Contable, Extractos y su tablero, Revisión, «marcá y te sugiero»,
  Analítica, informe nuevo, tabla de 6 ediciones.
- Extractos: la banda muestra DEXIAE Contable en vez de CORE.
- Demo /app con la UI 2.8.0: extractos, analítica y revisión (antes faltaban),
  recorrido por Extractos, Excels de ejemplo regenerados.
- Contable paga por Mercado Pago (fundador mensual 59.000 y anual 565.000).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/app/ejemplos/DEXIAE_ejemplo_extraccion.xlsx
+++ b/app/ejemplos/DEXIAE_ejemplo_extraccion.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validación" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validación detalle" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revisión" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Validación'!$A$8:$J$10</definedName>
@@ -88,7 +89,7 @@
       <u val="single"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -120,8 +121,13 @@
         <fgColor rgb="00EDE9FE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF7E0"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="20">
+  <borders count="22">
     <border>
       <left/>
       <right/>
@@ -300,11 +306,35 @@
         <color rgb="00E2E8F0"/>
       </bottom>
     </border>
+    <border>
+      <left style="thick">
+        <color rgb="002563EB"/>
+      </left>
+      <right style="thin">
+        <color rgb="00E2E8F0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00E2E8F0"/>
+      </top>
+      <bottom/>
+    </border>
+    <border>
+      <left style="thick">
+        <color rgb="0094A3B8"/>
+      </left>
+      <right style="thin">
+        <color rgb="00E2E8F0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00E2E8F0"/>
+      </top>
+      <bottom/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -384,6 +414,14 @@
     <xf numFmtId="0" fontId="7" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -458,6 +496,21 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>DEXIAE</author>
+  </authors>
+  <commentList>
+    <comment ref="F9" authorId="0" shapeId="0">
+      <text>
+        <t>Sin revisar: «TOTAL» es obligatorio y no se leyó nada.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -749,7 +802,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -788,21 +841,6 @@
           <t>ESTADO_PROCESO</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>VALIDACION</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>VALIDACION_DETALLE</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>VALIDACION_NIVEL</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -840,16 +878,6 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -887,16 +915,6 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -934,16 +952,6 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -981,21 +989,6 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>1 hallazgo(s)</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>CUIT inválido (dígito verificador): 30111111119</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1033,16 +1026,6 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1080,16 +1063,6 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1127,16 +1100,6 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1164,19 +1127,10 @@
           <t>0001-00001238</t>
         </is>
       </c>
+      <c r="F9" s="31" t="n"/>
       <c r="G9" t="inlineStr">
         <is>
           <t>DATOS FALTANTES</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>OK</t>
         </is>
       </c>
     </row>
@@ -1216,16 +1170,6 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1263,24 +1207,10 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>1 hallazgo(s)</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>Duplicado lógico: CUIT+NUMERO repetido (igual que FC_DEMO_003.pdf)</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
-        </is>
-      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -1320,20 +1250,20 @@
       </c>
     </row>
     <row r="3" ht="26" customHeight="1">
-      <c r="A3" s="4" t="n">
+      <c r="A3" s="32" t="n">
         <v>2</v>
       </c>
       <c r="B3" s="5" t="n"/>
       <c r="C3" s="5" t="n"/>
       <c r="D3" s="6" t="n"/>
-      <c r="E3" s="4" t="n">
+      <c r="E3" s="32" t="n">
         <v>2</v>
       </c>
       <c r="F3" s="6" t="n"/>
       <c r="G3" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="H3" s="7" t="n">
+      <c r="H3" s="33" t="n">
         <v>0</v>
       </c>
       <c r="I3" s="6" t="n"/>
@@ -1371,24 +1301,13 @@
           <t>DUPLICIDAD · más de uno donde va uno solo</t>
         </is>
       </c>
-      <c r="B5" s="13" t="n"/>
-      <c r="C5" s="13" t="n"/>
-      <c r="D5" s="13" t="n"/>
       <c r="E5" s="14" t="inlineStr">
         <is>
           <t>VALOR NO VÁLIDO · el dato no cumple la condición de la regla</t>
         </is>
       </c>
-      <c r="F5" s="15" t="n"/>
-    </row>
-    <row r="6" ht="4" customHeight="1">
-      <c r="A6" s="13" t="n"/>
-      <c r="B6" s="13" t="n"/>
-      <c r="C6" s="13" t="n"/>
-      <c r="D6" s="13" t="n"/>
-      <c r="E6" s="15" t="n"/>
-      <c r="F6" s="15" t="n"/>
-    </row>
+    </row>
+    <row r="6" ht="4" customHeight="1"/>
     <row r="7" ht="6" customHeight="1"/>
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="16" t="inlineStr">
@@ -1818,4 +1737,116 @@
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="34" t="inlineStr">
+        <is>
+          <t>HORA (UTC)</t>
+        </is>
+      </c>
+      <c r="B1" s="34" t="inlineStr">
+        <is>
+          <t>USUARIO</t>
+        </is>
+      </c>
+      <c r="C1" s="34" t="inlineStr">
+        <is>
+          <t>EQUIPO</t>
+        </is>
+      </c>
+      <c r="D1" s="34" t="inlineStr">
+        <is>
+          <t>DOCUMENTO</t>
+        </is>
+      </c>
+      <c r="E1" s="34" t="inlineStr">
+        <is>
+          <t>CAMPO / REGLA</t>
+        </is>
+      </c>
+      <c r="F1" s="34" t="inlineStr">
+        <is>
+          <t>DECISIÓN</t>
+        </is>
+      </c>
+      <c r="G1" s="34" t="inlineStr">
+        <is>
+          <t>SE LEYÓ</t>
+        </is>
+      </c>
+      <c r="H1" s="34" t="inlineStr">
+        <is>
+          <t>EN EL EXCEL</t>
+        </is>
+      </c>
+      <c r="I1" s="34" t="inlineStr">
+        <is>
+          <t>NOTA</t>
+        </is>
+      </c>
+      <c r="J1" s="34" t="inlineStr">
+        <is>
+          <t>HUELLA</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Cabeza de la cadena</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>(sin decisiones)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Qué prueba</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Trazabilidad local: detecta que se editó o se sacó una decisión de la base. Usuario y equipo son la sesión de Windows que decidió, no una firma.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Sin terminar</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Se generó con 1 caso(s) sin decidir, marcados en su hoja.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>